<commit_message>
chore: remove Swagger UI and OpenAPI documentation (1.6MB binary saving)
Swagger UI was bundled into the binary via include_str! macros but had
no UI entry point — users could never reach it. Pure dead weight.

Deleted:
- src-tauri/static/swagger-ui/ (swagger-ui-bundle.js, swagger-ui.css, favicon.ico)
- src-tauri/static/openapi.json

Removed from Rust:
- gateway_routes.rs: handle_openapi_route, handle_docs_root_route,
  handle_static_asset functions and their tests
- gateway_routes.rs: simplify handle_unknown_route (remove whitelist)
- proxy.rs: remove /openapi.json and / swagger routes from match block
- proxy.rs: remove swagger paths from CORS whitelists
- server/tests.rs: update whitelist test arrays

handle_models_route and handle_unknown_route are preserved — they
serve the /models endpoint used by external API consumers.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AX_STUDIO_FEATURE_INVENTORY.xlsx
+++ b/docs/AX_STUDIO_FEATURE_INVENTORY.xlsx
@@ -7,6 +7,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removal Tracker" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Status" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OpenClaw Comparison" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Inventory'!$A$1:$H$1</definedName>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -83,8 +84,13 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -151,6 +157,21 @@
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border/>
@@ -186,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -278,6 +299,24 @@
     <xf numFmtId="0" fontId="10" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14486,4 +14525,2316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="17" min="1" max="1"/>
+    <col width="32" customWidth="1" style="17" min="2" max="2"/>
+    <col width="22" customWidth="1" style="17" min="3" max="3"/>
+    <col width="22" customWidth="1" style="17" min="4" max="4"/>
+    <col width="14" customWidth="1" style="17" min="5" max="5"/>
+    <col width="22" customWidth="1" style="17" min="6" max="6"/>
+    <col width="50" customWidth="1" style="17" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="17">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>AX Studio vs OpenClaw — Feature Comparison &amp; Migration Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="17">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>Migration Action</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="17">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Multi-thread chat</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>✅ Rich Tauri UI</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>✅ Terminal + 25 channels</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F3" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Remove AX version</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw connects WhatsApp, Telegram, Discord, Slack, iMessage etc. AX Studio is desktop-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="17">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Streaming responses</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>✅ AI SDK 5</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>✅ Block streaming</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F4" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep both</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Both work well — no action needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="17">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Memory (@remember/@forget)</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>✅ Basic key-value</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>✅ LanceDB vector DB</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Remove AX version</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw uses LanceDB with vector embeddings — much more powerful</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="17">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Thread search (FZF/Fuse)</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>✅ FZF + Fuse.js</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>✅ Built-in</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F6" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Both have search</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="17">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Thread export</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>✅ JSON/CSV/JSONL</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Unique to AX Studio — useful for data portability</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="17">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Chat &amp; Messaging</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Pinned threads</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>UI convenience feature</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="17">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E9" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has more complete implementation with failover and auth rotation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="17">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E10" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has more complete implementation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="17">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Google Gemini</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has more complete implementation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="17">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Azure OpenAI</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw covers this</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="17">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>OpenRouter</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E13" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw covers this</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="17">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw covers this</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="17">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>❌ Removed</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>N/A — already removed</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Already removed from AX Studio. OpenClaw has it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="17">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>HuggingFace Inference</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio unique — open-source model access</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>➕ Add or use OpenClaw</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>Strong coding models — OpenClaw has it</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="17">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Together AI / Fireworks</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has 20+ providers vs our 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="17">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>AWS Bedrock</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Enterprise provider — OpenClaw has it</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="17">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>AI Providers</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Ollama / LM Studio</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>✅ Via Custom URL</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>✅ Native</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep custom URL</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio handles this via custom OpenAI-compatible URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="17">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>llama.cpp native</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>✅ Full plugin</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>❌ Via Ollama only</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio's biggest differentiator. GPU Metal/CUDA, GGUF loading, 40+ engine params</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="17">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>GGUF model loading</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F22" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Direct GGUF file loading — not possible in OpenClaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="17">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>GPU/Metal acceleration</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G23" s="20" t="inlineStr">
+        <is>
+          <t>Hardware GPU offloading, flash attention, split mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="17">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Model Hub (HuggingFace)</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>✅ Full browser+download</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E24" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F24" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>Browse HuggingFace catalog, download GGUF files with resume + SHA256 verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="17">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>Engine settings (40+ params)</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>Context size, GPU layers, temperature, etc — full control</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="17">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Local Inference</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Backend auto-update</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E26" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F26" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>Auto-download llama.cpp binary updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="17">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>MCP server management UI</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>✅ Full UI</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>✅ Via mcporter (minimal)</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F27" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Better UI</t>
+        </is>
+      </c>
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio has full add/edit/delete/rename UI. OpenClaw's mcporter is bridge-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="17">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Tool execution</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E28" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F28" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G28" s="20" t="inlineStr">
+        <is>
+          <t>Both handle tool execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="17">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="inlineStr">
+        <is>
+          <t>Tool approval workflow</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>✅ Per-tool UI</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>Per-tool approval dialog, global/per-tool permissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="17">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>MCP auto-restart</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>✅ Exponential backoff</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E30" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP</t>
+        </is>
+      </c>
+      <c r="G30" s="20" t="inlineStr">
+        <is>
+          <t>Server crash recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="17">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>Default MCP servers</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>✅ Exa, sequential-think</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>✅ More options</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F31" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G31" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has more default MCP integrations</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="17">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>RAG &amp; Knowledge</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Document upload/chunking</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>✅ PDF, MD, text</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>✅ PDF, images, multi-format</t>
+        </is>
+      </c>
+      <c r="E32" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F32" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G32" s="20" t="inlineStr">
+        <is>
+          <t>Both handle documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="17">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>RAG &amp; Knowledge</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>Vector search</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>✅ AkiDB (custom)</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>✅ LanceDB (mature)</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Migrate to LanceDB</t>
+        </is>
+      </c>
+      <c r="G33" s="20" t="inlineStr">
+        <is>
+          <t>LanceDB is battle-tested. AkiDB is custom-built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="17">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>RAG &amp; Knowledge</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Web search</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>✅ Exa + DDG</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>✅ Brave+DDG+Tavily+Exa+Firecrawl</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F34" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G34" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has significantly more search providers</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="17">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>RAG &amp; Knowledge</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>Web scraping</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>✅ Basic (scraper.rs)</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>✅ Firecrawl advanced</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G35" s="20" t="inlineStr">
+        <is>
+          <t>Firecrawl is more powerful than our basic scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="17">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>RAG &amp; Knowledge</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>AkiDB knowledge base</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>✅ Custom fabric-ingest</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E36" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F36" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP for now</t>
+        </is>
+      </c>
+      <c r="G36" s="20" t="inlineStr">
+        <is>
+          <t>Evaluate replacing with LanceDB during migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="17">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>Agent orchestration</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
+        <is>
+          <t>✅ Router/Seq/Parallel</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>✅ Full RPC runtime</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F37" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G37" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw's RPC runtime is more sophisticated with workspace isolation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="17">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="inlineStr">
+        <is>
+          <t>Agent skills/plugins</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>✅ 4 extensions</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>✅ 67 built-in skills</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F38" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G38" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw has 67 skills: Spotify, Notion, 1Password, GitHub, smart home etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="17">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>Agent cost estimation</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F39" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep for now</t>
+        </is>
+      </c>
+      <c r="G39" s="20" t="inlineStr">
+        <is>
+          <t>Useful feature, evaluate during migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="17">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Agent run logs</t>
+        </is>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E40" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F40" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep for now</t>
+        </is>
+      </c>
+      <c r="G40" s="20" t="inlineStr">
+        <is>
+          <t>Debugging tool — keep until migrated</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="17">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="inlineStr">
+        <is>
+          <t>Team builder UI</t>
+        </is>
+      </c>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>✅ Visual builder</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>❌ Code/config based</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Better UX</t>
+        </is>
+      </c>
+      <c r="G41" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio's visual agent team builder is more user-friendly</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="17">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="inlineStr">
+        <is>
+          <t>Sub-agent routing</t>
+        </is>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="inlineStr">
+        <is>
+          <t>✅ Registry-backed</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F42" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G42" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw's registry-backed routing is more powerful</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="17">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>Speech-to-Text</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>❌ Removed</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="inlineStr">
+        <is>
+          <t>✅ Whisper/Deepgram</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>➕ Add from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>We removed STT — OpenClaw has full Whisper + Deepgram integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="17">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Text-to-Speech</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>❌ Removed</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="inlineStr">
+        <is>
+          <t>✅ ElevenLabs/edge-tts</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>➕ Add from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G44" s="20" t="inlineStr">
+        <is>
+          <t>We removed TTS — OpenClaw has ElevenLabs, MLX, edge-tts</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="17">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Wake words</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>✅ macOS/iOS</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>➕ Add from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G45" s="20" t="inlineStr">
+        <is>
+          <t>Hands-free activation</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="17">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="inlineStr">
+        <is>
+          <t>Continuous voice</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D46" s="21" t="inlineStr">
+        <is>
+          <t>✅ Android/iOS</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>➕ Add from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G46" s="20" t="inlineStr">
+        <is>
+          <t>Real-time voice conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="17">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>Linear/Notion/Slack/Jira</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>✅ OAuth + MCP</t>
+        </is>
+      </c>
+      <c r="D47" s="21" t="inlineStr">
+        <is>
+          <t>✅ Via skills</t>
+        </is>
+      </c>
+      <c r="E47" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F47" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G47" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw integrations are more complete via skills ecosystem</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="17">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Multi-channel messaging</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D48" s="21" t="inlineStr">
+        <is>
+          <t>✅ 25+ channels</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>➕ Get from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G48" s="20" t="inlineStr">
+        <is>
+          <t>WhatsApp, Telegram, Discord, iMessage etc. — massive advantage</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="17">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="inlineStr">
+        <is>
+          <t>GitHub integration</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>➕ Get from OpenClaw</t>
+        </is>
+      </c>
+      <c r="G49" s="20" t="inlineStr">
+        <is>
+          <t>GitHub + Issues skill in OpenClaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="17">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>UI &amp; Artifacts</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>Artifacts engine</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>✅ HTML/React/SVG/Vega</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E50" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G50" s="20" t="inlineStr">
+        <is>
+          <t>Sandboxed iframe rendering of HTML, React, ChartJS, Vega artifacts — no equivalent in OpenClaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1" s="17">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>UI &amp; Artifacts</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Reasoning display</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E51" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F51" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G51" s="20" t="inlineStr">
+        <is>
+          <t>Both support thinking/reasoning blocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1" s="17">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>UI &amp; Artifacts</t>
+        </is>
+      </c>
+      <c r="B52" s="20" t="inlineStr">
+        <is>
+          <t>Desktop UI (Tauri)</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>✅ Polished</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>✅ Terminal-first</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F52" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Core value</t>
+        </is>
+      </c>
+      <c r="G52" s="20" t="inlineStr">
+        <is>
+          <t>AX Studio's polished Tauri UI is a key differentiator vs terminal-first OpenClaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1" s="17">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>UI &amp; Artifacts</t>
+        </is>
+      </c>
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>Canvas/Agent-driven UI</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>✅ A2UI Canvas</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>OpenClaw</t>
+        </is>
+      </c>
+      <c r="F53" s="24" t="inlineStr">
+        <is>
+          <t>➕ Consider adding</t>
+        </is>
+      </c>
+      <c r="G53" s="20" t="inlineStr">
+        <is>
+          <t>OpenClaw's Canvas allows agent-controlled interactive UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="17">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>Hardware &amp; System</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>Hardware monitor</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>✅ GPU/CPU/RAM</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP — Unique</t>
+        </is>
+      </c>
+      <c r="G54" s="20" t="inlineStr">
+        <is>
+          <t>Critical for local inference — GPU device management, NVIDIA/Vulkan detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="17">
+      <c r="A55" s="20" t="inlineStr">
+        <is>
+          <t>Hardware &amp; System</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="inlineStr">
+        <is>
+          <t>System monitor</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F55" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G55" s="20" t="inlineStr">
+        <is>
+          <t>Separate floating window</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1" s="17">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>Hardware &amp; System</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>App updates (HMAC)</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E56" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F56" s="38" t="inlineStr">
+        <is>
+          <t>🟠 Use OpenClaw's</t>
+        </is>
+      </c>
+      <c r="G56" s="20" t="inlineStr">
+        <is>
+          <t>Both have update checking</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1" s="17">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>Hardware &amp; System</t>
+        </is>
+      </c>
+      <c r="B57" s="20" t="inlineStr">
+        <is>
+          <t>Factory reset</t>
+        </is>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E57" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F57" s="29" t="inlineStr">
+        <is>
+          <t>✅ Keep</t>
+        </is>
+      </c>
+      <c r="G57" s="20" t="inlineStr">
+        <is>
+          <t>User data management</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1" s="17">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>Path traversal prevention</t>
+        </is>
+      </c>
+      <c r="C58" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>✅ SSRF-guarded</t>
+        </is>
+      </c>
+      <c r="E58" s="39" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="F58" s="40" t="inlineStr">
+        <is>
+          <t>✅ Keep both</t>
+        </is>
+      </c>
+      <c r="G58" s="20" t="inlineStr">
+        <is>
+          <t>Both have security safeguards</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1" s="17">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>MCP process whitelist</t>
+        </is>
+      </c>
+      <c r="C59" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E59" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F59" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP</t>
+        </is>
+      </c>
+      <c r="G59" s="20" t="inlineStr">
+        <is>
+          <t>Only allows node/python/bun/npx/uvx — important security feature</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1" s="17">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="inlineStr">
+        <is>
+          <t>Constant-time auth</t>
+        </is>
+      </c>
+      <c r="C60" s="21" t="inlineStr">
+        <is>
+          <t>✅ subtle crate</t>
+        </is>
+      </c>
+      <c r="D60" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E60" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F60" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP</t>
+        </is>
+      </c>
+      <c r="G60" s="20" t="inlineStr">
+        <is>
+          <t>Timing-safe proxy API key comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1" s="17">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>SHA256 download verify</t>
+        </is>
+      </c>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" s="23" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="E61" s="29" t="inlineStr">
+        <is>
+          <t>AX Studio</t>
+        </is>
+      </c>
+      <c r="F61" s="29" t="inlineStr">
+        <is>
+          <t>✅ KEEP</t>
+        </is>
+      </c>
+      <c r="G61" s="20" t="inlineStr">
+        <is>
+          <t>All model downloads SHA256-verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1" s="17">
+      <c r="A64" s="42" t="inlineStr">
+        <is>
+          <t>MIGRATION SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="35" t="inlineStr">
+        <is>
+          <t>✅ KEEP in AX Studio (Unique value)</t>
+        </is>
+      </c>
+      <c r="B65" s="20" t="inlineStr">
+        <is>
+          <t>llama.cpp local inference, Model Hub, Artifacts Engine, MCP UI, Hardware Monitor, Team Builder UI, Security features</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="43" t="inlineStr">
+        <is>
+          <t>🟠 Remove / Replace with OpenClaw</t>
+        </is>
+      </c>
+      <c r="B66" s="20" t="inlineStr">
+        <is>
+          <t>Provider management, Agent orchestration core, Memory (use LanceDB), Web search (use Firecrawl), Multi-channel messaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="33" t="inlineStr">
+        <is>
+          <t>➕ Gain from OpenClaw base</t>
+        </is>
+      </c>
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>Voice (STT/TTS/wake words), 20+ AI providers, 67 skills ecosystem, Multi-channel (WhatsApp/Telegram/Discord), GitHub integration, Canvas A2UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="44" t="inlineStr">
+        <is>
+          <t>Tie — both cover equally</t>
+        </is>
+      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>Streaming, thread search, document upload, reasoning display, security safeguards</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B66:G66"/>
+    <mergeCell ref="B67:G67"/>
+    <mergeCell ref="B65:G65"/>
+    <mergeCell ref="B68:G68"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>